<commit_message>
Add security test report and updated RTM, Closes #9, Closes #13
</commit_message>
<xml_diff>
--- a/docs/RTM/Test_Cases_HMS.xlsx
+++ b/docs/RTM/Test_Cases_HMS.xlsx
@@ -1489,7 +1489,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J20" s="23" t="n"/>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>#17</t>
+        </is>
+      </c>
       <c r="K20" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>
@@ -1601,7 +1605,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J22" s="23" t="n"/>
+      <c r="J22" s="23" t="inlineStr">
+        <is>
+          <t>#18</t>
+        </is>
+      </c>
       <c r="K22" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>
@@ -1657,7 +1665,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J23" s="23" t="n"/>
+      <c r="J23" s="23" t="inlineStr">
+        <is>
+          <t>#18</t>
+        </is>
+      </c>
       <c r="K23" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>
@@ -2201,7 +2213,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J33" s="23" t="n"/>
+      <c r="J33" s="23" t="inlineStr">
+        <is>
+          <t>#19</t>
+        </is>
+      </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>
@@ -2817,7 +2833,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J44" s="23" t="n"/>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>#20</t>
+        </is>
+      </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>
@@ -3145,7 +3165,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J50" s="23" t="n"/>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
+          <t>#22</t>
+        </is>
+      </c>
       <c r="K50" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>
@@ -3425,7 +3449,11 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="J55" s="23" t="n"/>
+      <c r="J55" s="23" t="inlineStr">
+        <is>
+          <t>#22</t>
+        </is>
+      </c>
       <c r="K55" s="23" t="inlineStr">
         <is>
           <t>Rohan Agarwal</t>

</xml_diff>